<commit_message>
feat(agent): add vol3 integrity grading harness
</commit_message>
<xml_diff>
--- a/docklive-inline-agent/samples/견적서양식.xlsx
+++ b/docklive-inline-agent/samples/견적서양식.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/857ba777ae50cf6d/바탕 화면/LiveDock/docklive-inline-agent/samples/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="11_4B48EDCF95615C5EE102E4B545B996382B4D9D6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6A1BA8F4-EA93-4469-A4F8-3C03E491917B}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_4B48EDCF95615C5EE102E4B545B996382B4D9D6C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0E3549E-180F-4CD5-9626-600212CD1DB2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>견 적 서</t>
   </si>
@@ -73,6 +73,15 @@
   </si>
   <si>
     <t>모니터암</t>
+  </si>
+  <si>
+    <t>노트북</t>
+  </si>
+  <si>
+    <t>모니터</t>
+  </si>
+  <si>
+    <t>키보드</t>
   </si>
 </sst>
 </file>
@@ -171,6 +180,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -458,7 +471,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:F14"/>
+  <dimension ref="B2:F17"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -528,61 +541,115 @@
     </row>
     <row r="10" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B10" s="3">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="3">
         <v>2</v>
       </c>
-      <c r="C10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="3">
-        <v>5</v>
-      </c>
       <c r="E10" s="3">
-        <v>42000</v>
+        <v>1200000</v>
       </c>
       <c r="F10" s="5">
-        <f>D10*E10</f>
-        <v>210000</v>
+        <f t="shared" ref="F10:F12" si="0">D10*E10</f>
+        <v>2400000</v>
       </c>
     </row>
     <row r="11" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B11" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D11" s="3">
         <v>3</v>
       </c>
       <c r="E11" s="3">
+        <v>350000</v>
+      </c>
+      <c r="F11" s="5">
+        <f t="shared" si="0"/>
+        <v>1050000</v>
+      </c>
+    </row>
+    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B12" s="3">
+        <v>3</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="3">
+        <v>5</v>
+      </c>
+      <c r="E12" s="3">
+        <v>45000</v>
+      </c>
+      <c r="F12" s="5">
+        <f t="shared" si="0"/>
+        <v>225000</v>
+      </c>
+    </row>
+    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B13" s="3">
+        <v>2</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="3">
+        <v>5</v>
+      </c>
+      <c r="E13" s="3">
+        <v>42000</v>
+      </c>
+      <c r="F13" s="5">
+        <f>D13*E13</f>
+        <v>210000</v>
+      </c>
+    </row>
+    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B14" s="3">
+        <v>3</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="3">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3">
         <v>89000</v>
       </c>
-      <c r="F11" s="5">
-        <f>D11*E11</f>
+      <c r="F14" s="5">
+        <f>D14*E14</f>
         <v>267000</v>
       </c>
     </row>
-    <row r="12" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="5"/>
-    </row>
-    <row r="13" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="5"/>
-    </row>
-    <row r="14" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="E14" s="4" t="s">
+    <row r="15" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="5"/>
+    </row>
+    <row r="16" spans="2:6" x14ac:dyDescent="0.3">
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="5"/>
+    </row>
+    <row r="17" spans="5:6" x14ac:dyDescent="0.3">
+      <c r="E17" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F14" s="5">
-        <f>SUM(F9:F13)</f>
-        <v>727000</v>
+      <c r="F17" s="5">
+        <f>SUM(F9:F16)</f>
+        <v>4402000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>